<commit_message>
Update example enrollment spreadsheet
</commit_message>
<xml_diff>
--- a/plantillas/ejemplos/solicitud-matricula-html-carga (2).xlsx
+++ b/plantillas/ejemplos/solicitud-matricula-html-carga (2).xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crrb\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\codex_projects\colegios\plantillas\ejemplos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF1A5B1C-A5C3-425F-A439-AF656658A4A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DF41AC1-F756-4DBD-AEC7-7D343C53AA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="123">
   <si>
     <t>Cedula</t>
   </si>
@@ -74,9 +74,6 @@
     <t>Fecha</t>
   </si>
   <si>
-    <t>0912345678</t>
-  </si>
-  <si>
     <t>Laura</t>
   </si>
   <si>
@@ -89,9 +86,6 @@
     <t>Perez</t>
   </si>
   <si>
-    <t>0991234567</t>
-  </si>
-  <si>
     <t>laura.gomez1@correo.com</t>
   </si>
   <si>
@@ -110,9 +104,6 @@
     <t>2026-03-01</t>
   </si>
   <si>
-    <t>0912345679</t>
-  </si>
-  <si>
     <t>Carlos</t>
   </si>
   <si>
@@ -122,9 +113,6 @@
     <t>Lopez</t>
   </si>
   <si>
-    <t>0991234568</t>
-  </si>
-  <si>
     <t>carlos.perez2@correo.com</t>
   </si>
   <si>
@@ -140,9 +128,6 @@
     <t>2026-03-02</t>
   </si>
   <si>
-    <t>0912345680</t>
-  </si>
-  <si>
     <t>Jose</t>
   </si>
   <si>
@@ -152,9 +137,6 @@
     <t>Mendoza</t>
   </si>
   <si>
-    <t>0991234569</t>
-  </si>
-  <si>
     <t>maria.torres3@correo.com</t>
   </si>
   <si>
@@ -173,9 +155,6 @@
     <t>2026-03-03</t>
   </si>
   <si>
-    <t>0912345681</t>
-  </si>
-  <si>
     <t>Jorge</t>
   </si>
   <si>
@@ -185,9 +164,6 @@
     <t>Garcia</t>
   </si>
   <si>
-    <t>0991234570</t>
-  </si>
-  <si>
     <t>jorge.ruiz4@correo.com</t>
   </si>
   <si>
@@ -206,9 +182,6 @@
     <t>2026-03-04</t>
   </si>
   <si>
-    <t>0912345682</t>
-  </si>
-  <si>
     <t>Ana</t>
   </si>
   <si>
@@ -221,9 +194,6 @@
     <t>Sanchez</t>
   </si>
   <si>
-    <t>0991234571</t>
-  </si>
-  <si>
     <t>ana.moreno5@correo.com</t>
   </si>
   <si>
@@ -242,9 +212,6 @@
     <t>2026-03-05</t>
   </si>
   <si>
-    <t>0912345683</t>
-  </si>
-  <si>
     <t>Luis</t>
   </si>
   <si>
@@ -254,9 +221,6 @@
     <t>Mora</t>
   </si>
   <si>
-    <t>0991234572</t>
-  </si>
-  <si>
     <t>luis.castro6@correo.com</t>
   </si>
   <si>
@@ -275,9 +239,6 @@
     <t>2026-03-06</t>
   </si>
   <si>
-    <t>0912345684</t>
-  </si>
-  <si>
     <t>Sofia</t>
   </si>
   <si>
@@ -287,9 +248,6 @@
     <t>Diaz</t>
   </si>
   <si>
-    <t>0991234573</t>
-  </si>
-  <si>
     <t>sofia.silva7@correo.com</t>
   </si>
   <si>
@@ -305,9 +263,6 @@
     <t>2026-03-07</t>
   </si>
   <si>
-    <t>0912345685</t>
-  </si>
-  <si>
     <t>Diego</t>
   </si>
   <si>
@@ -320,9 +275,6 @@
     <t>Ortega</t>
   </si>
   <si>
-    <t>0991234574</t>
-  </si>
-  <si>
     <t>diego.rojas8@correo.com</t>
   </si>
   <si>
@@ -338,9 +290,6 @@
     <t>2026-03-08</t>
   </si>
   <si>
-    <t>0912345686</t>
-  </si>
-  <si>
     <t>Paula</t>
   </si>
   <si>
@@ -350,9 +299,6 @@
     <t>Nunez</t>
   </si>
   <si>
-    <t>0991234575</t>
-  </si>
-  <si>
     <t>paula.vega9@correo.com</t>
   </si>
   <si>
@@ -365,18 +311,12 @@
     <t>2026-03-09</t>
   </si>
   <si>
-    <t>0912345687</t>
-  </si>
-  <si>
     <t>Gabriel</t>
   </si>
   <si>
     <t>Herrera</t>
   </si>
   <si>
-    <t>0991234576</t>
-  </si>
-  <si>
     <t>mateo.lopez10@correo.com</t>
   </si>
   <si>
@@ -420,6 +360,36 @@
   </si>
   <si>
     <t>El placeholder de la plantilla debe coincidir exactamente con el nombre de la columna del Excel.</t>
+  </si>
+  <si>
+    <t>0969019242</t>
+  </si>
+  <si>
+    <t>0969019243</t>
+  </si>
+  <si>
+    <t>0969019244</t>
+  </si>
+  <si>
+    <t>0969019245</t>
+  </si>
+  <si>
+    <t>0969019246</t>
+  </si>
+  <si>
+    <t>0969019247</t>
+  </si>
+  <si>
+    <t>0969019248</t>
+  </si>
+  <si>
+    <t>0969019249</t>
+  </si>
+  <si>
+    <t>0969019210</t>
+  </si>
+  <si>
+    <t>0969019211</t>
   </si>
 </sst>
 </file>
@@ -455,8 +425,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -797,9 +768,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="16.875" customWidth="1"/>
+    <col min="1" max="1" width="16.875" style="1" customWidth="1"/>
+    <col min="2" max="3" width="16.875" customWidth="1"/>
     <col min="4" max="4" width="18.875" customWidth="1"/>
     <col min="5" max="6" width="16.875" customWidth="1"/>
     <col min="7" max="7" width="23.75" bestFit="1" customWidth="1"/>
@@ -809,8 +781,8 @@
     <col min="15" max="17" width="16.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -862,27 +834,27 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B2" t="s">
         <v>17</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>18</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>19</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>20</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="G2" t="s">
         <v>21</v>
-      </c>
-      <c r="F2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G2" t="s">
-        <v>23</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -897,45 +869,45 @@
         <v>1701</v>
       </c>
       <c r="L2" t="s">
+        <v>22</v>
+      </c>
+      <c r="M2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O2" t="s">
         <v>24</v>
       </c>
-      <c r="M2" t="s">
+      <c r="P2" t="s">
         <v>25</v>
       </c>
-      <c r="N2" t="s">
-        <v>21</v>
-      </c>
-      <c r="O2" t="s">
+      <c r="Q2" t="s">
         <v>26</v>
       </c>
-      <c r="P2" t="s">
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B3" t="s">
         <v>27</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="C3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="D3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" t="s">
         <v>29</v>
       </c>
-      <c r="B3" t="s">
+      <c r="F3" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="G3" t="s">
         <v>30</v>
-      </c>
-      <c r="C3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G3" t="s">
-        <v>34</v>
       </c>
       <c r="H3">
         <v>1</v>
@@ -950,45 +922,45 @@
         <v>1701</v>
       </c>
       <c r="L3" t="s">
+        <v>31</v>
+      </c>
+      <c r="M3" t="s">
+        <v>32</v>
+      </c>
+      <c r="N3" t="s">
+        <v>19</v>
+      </c>
+      <c r="O3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P3" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
         <v>35</v>
       </c>
-      <c r="M3" t="s">
+      <c r="D4" t="s">
         <v>36</v>
       </c>
-      <c r="N3" t="s">
-        <v>20</v>
-      </c>
-      <c r="O3" t="s">
+      <c r="E4" t="s">
         <v>37</v>
       </c>
-      <c r="P3" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q3" t="s">
+      <c r="F4" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="G4" t="s">
         <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E4" t="s">
-        <v>42</v>
-      </c>
-      <c r="F4" t="s">
-        <v>43</v>
-      </c>
-      <c r="G4" t="s">
-        <v>44</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -1003,45 +975,45 @@
         <v>1701</v>
       </c>
       <c r="L4" t="s">
+        <v>39</v>
+      </c>
+      <c r="M4" t="s">
+        <v>40</v>
+      </c>
+      <c r="N4" t="s">
+        <v>41</v>
+      </c>
+      <c r="O4" t="s">
+        <v>42</v>
+      </c>
+      <c r="P4" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" t="s">
         <v>45</v>
       </c>
-      <c r="M4" t="s">
+      <c r="D5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E5" t="s">
         <v>46</v>
       </c>
-      <c r="N4" t="s">
+      <c r="F5" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="G5" t="s">
         <v>47</v>
-      </c>
-      <c r="O4" t="s">
-        <v>48</v>
-      </c>
-      <c r="P4" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>50</v>
-      </c>
-      <c r="B5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E5" t="s">
-        <v>53</v>
-      </c>
-      <c r="F5" t="s">
-        <v>54</v>
-      </c>
-      <c r="G5" t="s">
-        <v>55</v>
       </c>
       <c r="H5">
         <v>1</v>
@@ -1056,45 +1028,45 @@
         <v>1701</v>
       </c>
       <c r="L5" t="s">
+        <v>48</v>
+      </c>
+      <c r="M5" t="s">
+        <v>49</v>
+      </c>
+      <c r="N5" t="s">
+        <v>50</v>
+      </c>
+      <c r="O5" t="s">
+        <v>51</v>
+      </c>
+      <c r="P5" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E6" t="s">
         <v>56</v>
       </c>
-      <c r="M5" t="s">
+      <c r="F6" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="G6" t="s">
         <v>57</v>
-      </c>
-      <c r="N5" t="s">
-        <v>58</v>
-      </c>
-      <c r="O5" t="s">
-        <v>59</v>
-      </c>
-      <c r="P5" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>61</v>
-      </c>
-      <c r="B6" t="s">
-        <v>62</v>
-      </c>
-      <c r="C6" t="s">
-        <v>63</v>
-      </c>
-      <c r="D6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E6" t="s">
-        <v>65</v>
-      </c>
-      <c r="F6" t="s">
-        <v>66</v>
-      </c>
-      <c r="G6" t="s">
-        <v>67</v>
       </c>
       <c r="H6">
         <v>1</v>
@@ -1109,45 +1081,45 @@
         <v>1701</v>
       </c>
       <c r="L6" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="M6" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="N6" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="O6" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="P6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="Q6" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>73</v>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>118</v>
       </c>
       <c r="B7" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="C7" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="D7" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="E7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F7" t="s">
-        <v>77</v>
+        <v>65</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="G7" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -1162,45 +1134,45 @@
         <v>1701</v>
       </c>
       <c r="L7" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="M7" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="N7" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="O7" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="P7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="Q7" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>84</v>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>119</v>
       </c>
       <c r="B8" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="C8" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="D8" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="E8" t="s">
-        <v>87</v>
-      </c>
-      <c r="F8" t="s">
-        <v>88</v>
+        <v>74</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="G8" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="H8">
         <v>1</v>
@@ -1215,45 +1187,45 @@
         <v>1701</v>
       </c>
       <c r="L8" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="M8" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="N8" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="O8" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="P8" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="Q8" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>94</v>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>120</v>
       </c>
       <c r="B9" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="C9" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="D9" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="E9" t="s">
-        <v>98</v>
-      </c>
-      <c r="F9" t="s">
-        <v>99</v>
+        <v>83</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="G9" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -1268,45 +1240,45 @@
         <v>1701</v>
       </c>
       <c r="L9" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="M9" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="N9" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="O9" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="P9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="Q9" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>105</v>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>121</v>
       </c>
       <c r="B10" t="s">
-        <v>106</v>
+        <v>89</v>
       </c>
       <c r="C10" t="s">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="D10" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="E10" t="s">
-        <v>108</v>
-      </c>
-      <c r="F10" t="s">
-        <v>109</v>
+        <v>91</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="G10" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
       <c r="H10">
         <v>1</v>
@@ -1321,45 +1293,45 @@
         <v>1701</v>
       </c>
       <c r="L10" t="s">
-        <v>111</v>
+        <v>93</v>
       </c>
       <c r="M10" t="s">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="N10" t="s">
+        <v>82</v>
+      </c>
+      <c r="O10" t="s">
+        <v>94</v>
+      </c>
+      <c r="P10" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" t="s">
+        <v>96</v>
+      </c>
+      <c r="D11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" t="s">
         <v>97</v>
       </c>
-      <c r="O10" t="s">
-        <v>112</v>
-      </c>
-      <c r="P10" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q10" t="s">
+      <c r="F11" s="1" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="11" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>114</v>
-      </c>
-      <c r="B11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" t="s">
-        <v>115</v>
-      </c>
-      <c r="D11" t="s">
-        <v>32</v>
-      </c>
-      <c r="E11" t="s">
-        <v>116</v>
-      </c>
-      <c r="F11" t="s">
-        <v>117</v>
-      </c>
       <c r="G11" t="s">
-        <v>118</v>
+        <v>98</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -1374,28 +1346,28 @@
         <v>1701</v>
       </c>
       <c r="L11" t="s">
-        <v>119</v>
+        <v>99</v>
       </c>
       <c r="M11" t="s">
-        <v>115</v>
+        <v>96</v>
       </c>
       <c r="N11" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="O11" t="s">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="P11" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="Q11" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:Q11" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:Q1 B2:E11 G2:Q11" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1403,55 +1375,55 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.875" customWidth="1"/>
     <col min="2" max="2" width="110.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>123</v>
+        <v>103</v>
       </c>
       <c r="B2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>125</v>
+        <v>105</v>
       </c>
       <c r="B3" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>127</v>
+        <v>107</v>
       </c>
       <c r="B4" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>129</v>
+        <v>109</v>
       </c>
       <c r="B5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>131</v>
+        <v>111</v>
       </c>
       <c r="B6" t="s">
-        <v>132</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>